<commit_message>
Add customer business analysis project
</commit_message>
<xml_diff>
--- a/Customer_Business_Analysis.xlsx
+++ b/Customer_Business_Analysis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ishit\Documents\Customer-Business-Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE3A330F-CCAD-453F-BB7C-444F37763EA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{80B2D2C3-71BA-4048-B485-71CFE3A0976F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="3" xr2:uid="{F1223D9D-EC31-4BBF-8218-8536B200EBD2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{F1223D9D-EC31-4BBF-8218-8536B200EBD2}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw Data" sheetId="1" r:id="rId1"/>
@@ -708,12 +708,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -725,6 +719,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -9131,58 +9131,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="24.6" x14ac:dyDescent="0.4">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="7"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="8" t="s">
         <v>136</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="8" t="s">
         <v>138</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="8" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="18" x14ac:dyDescent="0.35">
-      <c r="A4" s="11">
+      <c r="A4" s="9">
         <f>Analysis!B3</f>
         <v>50</v>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="9">
         <f>Analysis!B4</f>
         <v>50</v>
       </c>
-      <c r="C4" s="12">
+      <c r="C4" s="10">
         <f>Analysis!B5</f>
         <v>294600</v>
       </c>
-      <c r="D4" s="12">
+      <c r="D4" s="10">
         <f>Analysis!B6</f>
         <v>84650</v>
       </c>
-      <c r="E4" s="13">
+      <c r="E4" s="11">
         <f>Analysis!B8</f>
         <v>0.28733876442634082</v>
       </c>
@@ -9227,7 +9227,7 @@
       <c r="B1" s="14"/>
     </row>
     <row r="3" spans="1:2" ht="18" x14ac:dyDescent="0.35">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="7" t="s">
         <v>171</v>
       </c>
     </row>
@@ -9277,7 +9277,7 @@
       </c>
     </row>
     <row r="10" spans="1:2" ht="18" x14ac:dyDescent="0.35">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="7" t="s">
         <v>175</v>
       </c>
     </row>

</xml_diff>